<commit_message>
cambios de principal y funcion modificar casos
</commit_message>
<xml_diff>
--- a/Datos/informacion_usuarios.xlsx
+++ b/Datos/informacion_usuarios.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,51 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>N° Caso</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nombre y Apellido</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Edad</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Género</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Peso (kg)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Altura (m)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Rasgos Físicos</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Zona (Argentina)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Datos Extra</t>
         </is>
@@ -465,15 +477,15 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Matías López</t>
+          <t>Matías Sánchez</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -481,116 +493,116 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>76.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="F2" t="n">
-        <v>1.86</v>
+        <v>1.76</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos celestes, tez clara</t>
+          <t>Pelo rapado, ojos marrones, tez morena</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>GBA Norte</t>
+          <t>NEA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un fénix en el cuello</t>
+          <t>Lleva anteojos de lectura y reloj</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Martín Ramírez</t>
+          <t>Paula Benítez</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>66.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>1.73</v>
+        <v>1.65</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos miel, tez clara</t>
+          <t>Pelo pelirrojo rizado, ojos celestes, tez morena</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>GBA Sur</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una constelación en la pierna</t>
+          <t>Tiene un tatuaje de un fénix en el brazo</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Florencia Romero</t>
+          <t>Santiago Benítez</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>56.8</v>
+        <v>92.7</v>
       </c>
       <c r="F4" t="n">
-        <v>1.51</v>
+        <v>1.84</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos verdes, tez clara</t>
+          <t>Pelo castaño lacio, ojos miel, tez pálida</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>Patagonia</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un león en el hombro</t>
+          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Matías Sánchez</t>
+          <t>Juan Flores</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -598,53 +610,53 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>72.3</v>
+        <v>69</v>
       </c>
       <c r="F5" t="n">
-        <v>1.76</v>
+        <v>1.85</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos marrones, tez morena</t>
+          <t>Pelo castaño oscuro rizado, ojos celestes, tez trigueña</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>GBA Norte</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Lleva anteojos de lectura y reloj</t>
+          <t>Tiene un tatuaje de una ola en la muñeca</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gonzalo Silva</t>
+          <t>Jesús Alvarez</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>No Binario</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>87.40000000000001</v>
+        <v>76</v>
       </c>
       <c r="F6" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos celestes, tez clara</t>
+          <t>Pelo castaño lacio, ojos celestes, tez trigueña</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -654,99 +666,99 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Usa ropa oversize en tonos oscuros</t>
+          <t>Usa gorra negra y auriculares</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Florencia Flores</t>
+          <t>Luis Gómez</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>78.3</v>
+        <v>82</v>
       </c>
       <c r="F7" t="n">
-        <v>1.56</v>
+        <v>1.68</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pelo negro corto, ojos verdes, tez pálida</t>
+          <t>Pelo castaño oscuro rizado, ojos verdes, tez morena</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>NOA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una frase inspiradora en el cuello</t>
+          <t>Viste saco elegante y botas</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paula Benítez</t>
+          <t>Martín Silva</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>1.65</v>
+        <v>1.78</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos celestes, tez morena</t>
+          <t>Pelo rapado, ojos verdes, tez trigueña</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>GBA Sur</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un fénix en el brazo</t>
+          <t>Tiene un tatuaje de un león en la pierna</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Santiago Benítez</t>
+          <t>Nicolás Medina</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -754,233 +766,233 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>92.7</v>
+        <v>76.8</v>
       </c>
       <c r="F9" t="n">
-        <v>1.84</v>
+        <v>1.72</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos miel, tez pálida</t>
+          <t>Pelo rubio ondulado, ojos oscuros, tez morena</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Patagonia</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
+          <t>Usa campera de jean y mochila</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Juan Flores</t>
+          <t>Ana Pérez</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>69</v>
+        <v>52.1</v>
       </c>
       <c r="F10" t="n">
-        <v>1.85</v>
+        <v>1.74</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos celestes, tez trigueña</t>
+          <t>Pelo rapado, ojos miel, tez morena</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>GBA Norte</t>
+          <t>NEA</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una ola en la muñeca</t>
+          <t>Sin accesorios particulares</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Gonzalo Acosta</t>
+          <t>Agustina Fernández</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>91.7</v>
+        <v>55.7</v>
       </c>
       <c r="F11" t="n">
-        <v>1.94</v>
+        <v>1.73</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos celestes, tez morena</t>
+          <t>Pelo pelirrojo rizado, ojos celestes, tez pálida</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>GBA Sur</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una frase inspiradora en la pierna</t>
+          <t>Tiene un tatuaje de una brújula en el hombro</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jesús Alvarez</t>
+          <t>Diego Cáceres</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No Binario</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>76</v>
+        <v>90.5</v>
       </c>
       <c r="F12" t="n">
-        <v>1.85</v>
+        <v>1.67</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos celestes, tez trigueña</t>
+          <t>Pelo rubio ondulado, ojos verdes, tez morena</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>GBA Oeste</t>
+          <t>NEA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Usa gorra negra y auriculares</t>
+          <t>Tiene un tatuaje de una frase inspiradora en la espalda</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Luis Gómez</t>
+          <t>Daniela Ramírez</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>82</v>
+        <v>77.7</v>
       </c>
       <c r="F13" t="n">
-        <v>1.68</v>
+        <v>1.57</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos verdes, tez morena</t>
+          <t>Pelo castaño lacio, ojos marrones, tez clara</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NOA</t>
+          <t>GBA Norte</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Viste saco elegante y botas</t>
+          <t>Lleva anteojos de lectura y reloj</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Martín Silva</t>
+          <t>Agustina Rodríguez</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>72.40000000000001</v>
+        <v>62</v>
       </c>
       <c r="F14" t="n">
-        <v>1.78</v>
+        <v>1.56</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos verdes, tez trigueña</t>
+          <t>Pelo pelirrojo rizado, ojos marrones, tez pálida</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>Provincia de Buenos Aires</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un león en la pierna</t>
+          <t>Tiene un tatuaje de figuras geométricas en la espalda</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nicolás Medina</t>
+          <t>Ezequiel Díaz</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -988,19 +1000,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>76.8</v>
+        <v>82</v>
       </c>
       <c r="F15" t="n">
-        <v>1.72</v>
+        <v>1.85</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pelo rubio ondulado, ojos oscuros, tez morena</t>
+          <t>Pelo rubio ondulado, ojos marrones, tez clara</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>Región Pampeana</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1011,54 +1023,54 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ana Pérez</t>
+          <t>Alejandro Rodríguez</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>52.1</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>1.74</v>
+        <v>1.93</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos miel, tez morena</t>
+          <t>Pelo castaño lacio, ojos verdes, tez clara</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>Patagonia</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Sin accesorios particulares</t>
+          <t>Usa gorra negra y auriculares</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Agustina Fernández</t>
+          <t>Julia Rojas</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1066,194 +1078,194 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>55.7</v>
+        <v>67.8</v>
       </c>
       <c r="F17" t="n">
-        <v>1.73</v>
+        <v>1.57</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos celestes, tez pálida</t>
+          <t>Pelo pelirrojo rizado, ojos oscuros, tez trigueña</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>Provincia de Buenos Aires</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una brújula en el hombro</t>
+          <t>Usa ropa oversize en tonos oscuros</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Diego Cáceres</t>
+          <t>Gabriela Ramírez</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>90.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>1.67</v>
+        <v>1.54</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pelo rubio ondulado, ojos verdes, tez morena</t>
+          <t>Pelo castaño oscuro rizado, ojos marrones, tez clara</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>NOA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una frase inspiradora en la espalda</t>
+          <t>Viste ropa deportiva y zapatillas</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Daniela Ramírez</t>
+          <t>Alejandro Flores</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.7</v>
+        <v>97.7</v>
       </c>
       <c r="F19" t="n">
-        <v>1.57</v>
+        <v>1.73</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos marrones, tez clara</t>
+          <t>Pelo rubio ondulado, ojos celestes, tez trigueña</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>GBA Norte</t>
+          <t>GBA Sur</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Lleva anteojos de lectura y reloj</t>
+          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Agustina Rodríguez</t>
+          <t>Jesús Romero</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>No Binario</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>62</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>1.56</v>
+        <v>1.55</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos marrones, tez pálida</t>
+          <t>Pelo castaño lacio, ojos verdes, tez trigueña</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Provincia de Buenos Aires</t>
+          <t>GBA Norte</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de figuras geométricas en la espalda</t>
+          <t>Lleva anteojos de lectura y reloj</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ezequiel Díaz</t>
+          <t>Rocío Suárez</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>82</v>
+        <v>60.3</v>
       </c>
       <c r="F21" t="n">
-        <v>1.85</v>
+        <v>1.56</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Pelo rubio ondulado, ojos marrones, tez clara</t>
+          <t>Pelo castaño oscuro rizado, ojos celestes, tez pálida</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Región Pampeana</t>
+          <t>Provincia de Buenos Aires</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Usa campera de jean y mochila</t>
+          <t>Viste ropa deportiva y zapatillas</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alejandro Rodríguez</t>
+          <t>Gonzalo López</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1261,38 +1273,38 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>83.59999999999999</v>
+        <v>76.7</v>
       </c>
       <c r="F22" t="n">
-        <v>1.93</v>
+        <v>1.66</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos verdes, tez clara</t>
+          <t>Pelo negro corto, ojos verdes, tez pálida</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Patagonia</t>
+          <t>NEA</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Usa gorra negra y auriculares</t>
+          <t>Tiene un tatuaje de una brújula en el brazo</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Julia Rojas</t>
+          <t>Lucía Medina</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1300,92 +1312,92 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>67.8</v>
+        <v>75</v>
       </c>
       <c r="F23" t="n">
-        <v>1.57</v>
+        <v>1.65</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos oscuros, tez trigueña</t>
+          <t>Pelo rubio ondulado, ojos miel, tez morena</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Provincia de Buenos Aires</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Usa ropa oversize en tonos oscuros</t>
+          <t>Tiene un tatuaje de una constelación en el brazo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Gabriela Ramírez</t>
+          <t>Ariel Sosa</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>No Binario</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>69.40000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="F24" t="n">
-        <v>1.54</v>
+        <v>1.78</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos marrones, tez clara</t>
+          <t>Pelo castaño oscuro rizado, ojos miel, tez morena</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NOA</t>
+          <t>GBA Oeste</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Viste ropa deportiva y zapatillas</t>
+          <t>Lleva anteojos de lectura y reloj</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alejandro Flores</t>
+          <t>Alex Cáceres</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>No Binario</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>97.7</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>1.73</v>
+        <v>1.61</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Pelo rubio ondulado, ojos celestes, tez trigueña</t>
+          <t>Pelo castaño oscuro rizado, ojos verdes, tez trigueña</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1395,60 +1407,60 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
+          <t>Lleva un colgante de plata y anillos</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jesús Romero</t>
+          <t>Javier Ramírez</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No Binario</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>83.59999999999999</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="F26" t="n">
-        <v>1.55</v>
+        <v>1.72</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Pelo castaño lacio, ojos verdes, tez trigueña</t>
+          <t>Pelo negro corto, ojos verdes, tez morena</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>GBA Norte</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Lleva anteojos de lectura y reloj</t>
+          <t>Lleva un colgante de plata y anillos</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rocío Suárez</t>
+          <t>Florencia Castro</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1456,116 +1468,116 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>60.3</v>
+        <v>58.4</v>
       </c>
       <c r="F27" t="n">
-        <v>1.56</v>
+        <v>1.77</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos celestes, tez pálida</t>
+          <t>Pelo pelirrojo rizado, ojos oscuros, tez trigueña</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Provincia de Buenos Aires</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Viste ropa deportiva y zapatillas</t>
+          <t>Viste saco elegante y botas</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gonzalo López</t>
+          <t>Elena Sosa</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>76.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>1.66</v>
+        <v>1.51</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pelo negro corto, ojos verdes, tez pálida</t>
+          <t>Pelo castaño oscuro rizado, ojos celestes, tez pálida</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>Patagonia</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una brújula en el brazo</t>
+          <t>Lleva un colgante de plata y anillos</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Lucía Medina</t>
+          <t>Ariel González</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>No Binario</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>75</v>
+        <v>79.8</v>
       </c>
       <c r="F29" t="n">
-        <v>1.65</v>
+        <v>1.63</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Pelo rubio ondulado, ojos miel, tez morena</t>
+          <t>Pelo castaño oscuro rizado, ojos oscuros, tez morena</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>Región Pampeana</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una constelación en el brazo</t>
+          <t>Tiene un tatuaje de un fénix en el hombro</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ariel Sosa</t>
+          <t>Guadalupe Giménez</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1573,116 +1585,116 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>78.3</v>
+        <v>84.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1.78</v>
+        <v>1.65</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos miel, tez morena</t>
+          <t>Pelo canoso lacio, ojos celestes, tez pálida</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>GBA Oeste</t>
+          <t>Región Pampeana</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Lleva anteojos de lectura y reloj</t>
+          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alex Cáceres</t>
+          <t>Laura Giménez</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No Binario</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>87.40000000000001</v>
+        <v>61.4</v>
       </c>
       <c r="F31" t="n">
-        <v>1.61</v>
+        <v>1.69</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos verdes, tez trigueña</t>
+          <t>Pelo canoso lacio, ojos oscuros, tez trigueña</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>GBA Sur</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Lleva un colgante de plata y anillos</t>
+          <t>Viste saco elegante y botas</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Javier Ramírez</t>
+          <t>Laura García</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>93.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="F32" t="n">
         <v>1.72</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Pelo negro corto, ojos verdes, tez morena</t>
+          <t>Pelo pelirrojo rizado, ojos miel, tez morena</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>NEA</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Lleva un colgante de plata y anillos</t>
+          <t>Tiene un tatuaje de una frase inspiradora en el hombro</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Florencia Castro</t>
+          <t>Micaela Gómez</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1690,38 +1702,38 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>58.4</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F33" t="n">
-        <v>1.77</v>
+        <v>1.69</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos oscuros, tez trigueña</t>
+          <t>Pelo rapado, ojos celestes, tez morena</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>GBA Oeste</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Viste saco elegante y botas</t>
+          <t>Usa campera de jean y mochila</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Elena Sosa</t>
+          <t>Agustina Ramírez</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1729,194 +1741,194 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>67.90000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F34" t="n">
-        <v>1.51</v>
+        <v>1.67</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos celestes, tez pálida</t>
+          <t>Pelo rapado, ojos oscuros, tez morena</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Patagonia</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Lleva un colgante de plata y anillos</t>
+          <t>Tiene un tatuaje de una ola en la muñeca</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ariel González</t>
+          <t>María Flores</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>No Binario</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>79.8</v>
+        <v>75.8</v>
       </c>
       <c r="F35" t="n">
-        <v>1.63</v>
+        <v>1.75</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos oscuros, tez morena</t>
+          <t>Pelo castaño oscuro rizado, ojos miel, tez morena</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Región Pampeana</t>
+          <t>GBA Sur</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un fénix en el hombro</t>
+          <t>Tiene un tatuaje de una brújula en la pierna</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Guadalupe Giménez</t>
+          <t>Sofía Suárez</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>No Binario</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>84.7</v>
+        <v>74</v>
       </c>
       <c r="F36" t="n">
-        <v>1.65</v>
+        <v>1.63</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Pelo canoso lacio, ojos celestes, tez pálida</t>
+          <t>Pelo canoso lacio, ojos oscuros, tez trigueña</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Región Pampeana</t>
+          <t>NOA</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de figuras geométricas en la pierna</t>
+          <t>Tiene un tatuaje de un león en la muñeca</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Laura Giménez</t>
+          <t>Javier Mansilla</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>61.4</v>
+        <v>91.3</v>
       </c>
       <c r="F37" t="n">
-        <v>1.69</v>
+        <v>1.79</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pelo canoso lacio, ojos oscuros, tez trigueña</t>
+          <t>Pelo negro corto, ojos oscuros, tez pálida</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>GBA Oeste</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Viste saco elegante y botas</t>
+          <t>Tiene un tatuaje de un león en el brazo</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Laura García</t>
+          <t>Nicolás Silva</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>68.2</v>
+        <v>76.2</v>
       </c>
       <c r="F38" t="n">
-        <v>1.72</v>
+        <v>1.73</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pelo pelirrojo rizado, ojos miel, tez morena</t>
+          <t>Pelo rubio ondulado, ojos verdes, tez morena</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NEA</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una frase inspiradora en el hombro</t>
+          <t>Usa gorra negra y auriculares</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Micaela Gómez</t>
+          <t>Laura Rodríguez</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1924,34 +1936,34 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>68.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="F39" t="n">
-        <v>1.69</v>
+        <v>1.59</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos celestes, tez morena</t>
+          <t>Pelo castaño oscuro rizado, ojos miel, tez pálida</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>GBA Oeste</t>
+          <t>Patagonia</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Usa campera de jean y mochila</t>
+          <t>Lleva un colgante de plata y anillos</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Agustina Ramírez</t>
+          <t>Joaquín Flores</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1959,42 +1971,42 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>73.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F40" t="n">
-        <v>1.67</v>
+        <v>1.74</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pelo rapado, ojos oscuros, tez morena</t>
+          <t>Pelo canoso lacio, ojos oscuros, tez morena</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cuyo</t>
+          <t>NOA</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una ola en la muñeca</t>
+          <t>Viste saco elegante y botas</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>María Flores</t>
+          <t>María Cáceres</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2002,14 +2014,14 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>75.8</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="F41" t="n">
-        <v>1.75</v>
+        <v>1.61</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Pelo castaño oscuro rizado, ojos miel, tez morena</t>
+          <t>Pelo rapado, ojos verdes, tez pálida</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2019,317 +2031,83 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de una brújula en la pierna</t>
+          <t>Lleva un colgante de plata y anillos</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sofía Suárez</t>
+          <t>Juan Burgos</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Femenino</t>
+          <t>Masculino</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F42" t="n">
-        <v>1.63</v>
+        <v>1.68</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Pelo canoso lacio, ojos oscuros, tez trigueña</t>
+          <t>Pelo rubio ondulado, ojos marrones, tez trigueña</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>NOA</t>
+          <t>Cuyo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Tiene un tatuaje de un león en la muñeca</t>
+          <t>Tiene un tatuaje de flores de loto en la espalda</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Javier Mansilla</t>
+          <t>Gabriela Benítez</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Masculino</t>
+          <t>Femenino</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>91.3</v>
+        <v>78.5</v>
       </c>
       <c r="F43" t="n">
-        <v>1.79</v>
+        <v>1.58</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Pelo negro corto, ojos oscuros, tez pálida</t>
+          <t>Pelo castaño oscuro rizado, ojos marrones, tez pálida</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>GBA Oeste</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
-        <is>
-          <t>Tiene un tatuaje de un león en el brazo</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>45</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Nicolás Silva</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>23</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Masculino</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Pelo rubio ondulado, ojos verdes, tez morena</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Cuyo</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Usa gorra negra y auriculares</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>46</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Laura Rodríguez</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>31</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Femenino</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>64</v>
-      </c>
-      <c r="F45" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Pelo castaño oscuro rizado, ojos miel, tez pálida</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Patagonia</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Lleva un colgante de plata y anillos</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>47</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Joaquín Flores</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>44</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Masculino</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>78.59999999999999</v>
-      </c>
-      <c r="F46" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Pelo canoso lacio, ojos oscuros, tez morena</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>NOA</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Viste saco elegante y botas</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>48</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>María Cáceres</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>43</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Femenino</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>70.09999999999999</v>
-      </c>
-      <c r="F47" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Pelo rapado, ojos verdes, tez pálida</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>GBA Sur</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Lleva un colgante de plata y anillos</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>49</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Juan Burgos</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>47</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Masculino</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>80</v>
-      </c>
-      <c r="F48" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Pelo rubio ondulado, ojos marrones, tez trigueña</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Cuyo</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>Tiene un tatuaje de flores de loto en la espalda</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>50</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Gabriela Benítez</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>34</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Femenino</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="F49" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Pelo castaño oscuro rizado, ojos marrones, tez pálida</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>CABA</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
         <is>
           <t>Usa ropa oversize en tonos oscuros</t>
         </is>

</xml_diff>

<commit_message>
Cambio de verificacion de agregar caso
</commit_message>
<xml_diff>
--- a/Datos/informacion_usuarios.xlsx
+++ b/Datos/informacion_usuarios.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2347,6 +2347,45 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>52</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Marta Colome</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>80</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Femenino</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>80</v>
+      </c>
+      <c r="F50" t="n">
+        <v>150</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>pelo blanco</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>catamarca</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>